<commit_message>
actualizar agosto y septiembre
</commit_message>
<xml_diff>
--- a/fitness_registro.xlsx
+++ b/fitness_registro.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tepjf-my.sharepoint.com/personal/marissa_martinezg_te_gob_mx/Documents/marissa.martinezg/Downloads/reto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="319" documentId="11_70DB4BDF8D9753F325A0235AB6AABCFDF034A14B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C13D9771-ABE4-4870-857F-9F9B5A96376B}"/>
+  <xr:revisionPtr revIDLastSave="829" documentId="11_70DB4BDF8D9753F325A0235AB6AABCFDF034A14B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B49661D-57B7-4D3F-B11A-BDF9897860EB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro" sheetId="1" r:id="rId1"/>
     <sheet name="Multas" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="119">
   <si>
     <t>REGISTRO DIARIO  (SI = realizo | NO = no realizo)</t>
   </si>
@@ -163,6 +164,234 @@
   </si>
   <si>
     <t>INC</t>
+  </si>
+  <si>
+    <t>Mart 14/07</t>
+  </si>
+  <si>
+    <t>Mie 15/07</t>
+  </si>
+  <si>
+    <t>Jue 16/07</t>
+  </si>
+  <si>
+    <t>Vie 17/07</t>
+  </si>
+  <si>
+    <t>Sab 18/07</t>
+  </si>
+  <si>
+    <t>Dom 19/07</t>
+  </si>
+  <si>
+    <t>Lun 20/07</t>
+  </si>
+  <si>
+    <t>Mart 21/07</t>
+  </si>
+  <si>
+    <t>Mie 22/07</t>
+  </si>
+  <si>
+    <t>Jue 23/07</t>
+  </si>
+  <si>
+    <t>Vie 24/07</t>
+  </si>
+  <si>
+    <t>Sab 25/07</t>
+  </si>
+  <si>
+    <t>Dom 26/07</t>
+  </si>
+  <si>
+    <t>Lun 27/07</t>
+  </si>
+  <si>
+    <t>Mart 28/07</t>
+  </si>
+  <si>
+    <t>Mie 29/07</t>
+  </si>
+  <si>
+    <t>Jue 30/07</t>
+  </si>
+  <si>
+    <t>Vie 31/07</t>
+  </si>
+  <si>
+    <t>Sab 01/08</t>
+  </si>
+  <si>
+    <t>Dom 02/08</t>
+  </si>
+  <si>
+    <t>Lun 03/08</t>
+  </si>
+  <si>
+    <t>Sab 08/08</t>
+  </si>
+  <si>
+    <t>Dom 09/08</t>
+  </si>
+  <si>
+    <t>Mart 04/08</t>
+  </si>
+  <si>
+    <t>Mie 05/08</t>
+  </si>
+  <si>
+    <t>Jue 06/08</t>
+  </si>
+  <si>
+    <t>Vie 07/08</t>
+  </si>
+  <si>
+    <t>Lun 10/08</t>
+  </si>
+  <si>
+    <t>Mart 11/08</t>
+  </si>
+  <si>
+    <t>Mie 12/08</t>
+  </si>
+  <si>
+    <t>Jue 13/08</t>
+  </si>
+  <si>
+    <t>Vie 14/08</t>
+  </si>
+  <si>
+    <t>Sab 15/08</t>
+  </si>
+  <si>
+    <t>Dom 16/08</t>
+  </si>
+  <si>
+    <t>Lun 17/08</t>
+  </si>
+  <si>
+    <t>Mart 18/08</t>
+  </si>
+  <si>
+    <t>Mie 19/08</t>
+  </si>
+  <si>
+    <t>Jue 20/08</t>
+  </si>
+  <si>
+    <t>Vie 21/08</t>
+  </si>
+  <si>
+    <t>Sab 22/08</t>
+  </si>
+  <si>
+    <t>Dom 23/08</t>
+  </si>
+  <si>
+    <t>Lun 24/08</t>
+  </si>
+  <si>
+    <t>Mart 25/08</t>
+  </si>
+  <si>
+    <t>Mie 26/08</t>
+  </si>
+  <si>
+    <t>Jue 27/08</t>
+  </si>
+  <si>
+    <t>Vie 28/08</t>
+  </si>
+  <si>
+    <t>Sab 29/08</t>
+  </si>
+  <si>
+    <t>Dom 30/08</t>
+  </si>
+  <si>
+    <t>Lun 31/08</t>
+  </si>
+  <si>
+    <t>Mart 01/09</t>
+  </si>
+  <si>
+    <t>Mie 02/09</t>
+  </si>
+  <si>
+    <t>Jue 03/09</t>
+  </si>
+  <si>
+    <t>Vie 04/09</t>
+  </si>
+  <si>
+    <t>Sab 05/09</t>
+  </si>
+  <si>
+    <t>Dom 06/09</t>
+  </si>
+  <si>
+    <t>Lun 07/09</t>
+  </si>
+  <si>
+    <t>Mart 08/09</t>
+  </si>
+  <si>
+    <t>Mie 09/09</t>
+  </si>
+  <si>
+    <t>Jue 10/09</t>
+  </si>
+  <si>
+    <t>Vie 11/09</t>
+  </si>
+  <si>
+    <t>Sab 12/09</t>
+  </si>
+  <si>
+    <t>Dom 13/09</t>
+  </si>
+  <si>
+    <t>Lun 14/09</t>
+  </si>
+  <si>
+    <t>Mart 15/09</t>
+  </si>
+  <si>
+    <t>Mie 16/09</t>
+  </si>
+  <si>
+    <t>Vie 18/09</t>
+  </si>
+  <si>
+    <t>Sab 19/09</t>
+  </si>
+  <si>
+    <t>Dom 20/09</t>
+  </si>
+  <si>
+    <t>Jue 17/09</t>
+  </si>
+  <si>
+    <t>Lun 21/09</t>
+  </si>
+  <si>
+    <t>Mart 22/09</t>
+  </si>
+  <si>
+    <t>Mie 23/09</t>
+  </si>
+  <si>
+    <t>Jue 24/09</t>
+  </si>
+  <si>
+    <t>Vie 25/09</t>
+  </si>
+  <si>
+    <t>Sab 26/09</t>
+  </si>
+  <si>
+    <t>Dom 27/09</t>
   </si>
 </sst>
 </file>
@@ -273,7 +502,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -307,11 +536,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -352,6 +590,15 @@
     <xf numFmtId="14" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -363,11 +610,193 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF276221"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -401,10 +830,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -692,53 +1117,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:CW9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="25" width="8" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="12" hidden="1" customWidth="1"/>
+    <col min="6" max="7" width="9.28515625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" hidden="1" customWidth="1"/>
+    <col min="10" max="14" width="9.28515625" hidden="1" customWidth="1"/>
+    <col min="15" max="25" width="8" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:101" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="16" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="15"/>
-      <c r="V1" s="15"/>
-      <c r="W1" s="15"/>
-      <c r="X1" s="15"/>
-      <c r="Y1" s="15"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="18"/>
+      <c r="S1" s="18"/>
+      <c r="T1" s="18"/>
+      <c r="U1" s="18"/>
+      <c r="V1" s="18"/>
+      <c r="W1" s="18"/>
+      <c r="X1" s="18"/>
+      <c r="Y1" s="18"/>
     </row>
-    <row r="2" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:101" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -814,8 +1239,236 @@
       <c r="Y2" s="11" t="s">
         <v>37</v>
       </c>
+      <c r="Z2" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA2" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD2" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE2" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AG2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH2" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI2" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ2" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK2" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL2" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM2" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="AN2" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AO2" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="AP2" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="AQ2" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="AR2" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="AS2" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="AT2" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="AU2" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="AV2" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW2" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="AX2" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="AY2" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ2" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA2" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="BB2" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="BC2" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="BD2" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="BE2" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="BF2" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="BG2" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="BH2" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="BI2" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="BJ2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="BK2" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL2" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="BM2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BN2" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="BO2" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="BP2" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="BQ2" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="BR2" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="BS2" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="BT2" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="BU2" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV2" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="BW2" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="BX2" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="BY2" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="BZ2" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="CA2" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="CB2" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="CC2" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="CD2" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="CE2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="CF2" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="CG2" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="CH2" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="CI2" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="CJ2" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="CK2" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="CL2" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="CM2" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="CN2" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="CO2" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="CP2" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="CQ2" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="CR2" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="CS2" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="CT2" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="CU2" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="CV2" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="CW2" s="11" t="s">
+        <v>118</v>
+      </c>
     </row>
-    <row r="3" spans="1:25" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:101" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -892,8 +1545,228 @@
       <c r="Y3" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="Z3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AM3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AN3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AO3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AP3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AT3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BC3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BD3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BE3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BF3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BG3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BH3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BI3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BK3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BL3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BM3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BN3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BP3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BQ3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BR3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BS3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BT3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BU3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BV3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BY3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BZ3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CB3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CC3" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CD3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CF3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CG3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CH3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CJ3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CK3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CL3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CM3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CN3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CO3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CP3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CQ3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CS3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CT3" s="22"/>
+      <c r="CU3" s="22"/>
+      <c r="CV3" s="22"/>
+      <c r="CW3" s="22"/>
     </row>
-    <row r="4" spans="1:25" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:101" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -967,9 +1840,231 @@
       <c r="X4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Y4" s="7"/>
+      <c r="Y4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z4" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA4" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB4" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC4" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD4" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AN4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AP4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AR4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BC4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BD4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BE4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BF4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BG4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BK4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BL4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BM4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BN4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BP4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BQ4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BR4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BS4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BT4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BU4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BV4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BY4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BZ4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CB4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CC4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CD4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CE4" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CF4" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CG4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CH4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI4" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CJ4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CK4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CL4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CM4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CN4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CO4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CP4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="CQ4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CS4" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CT4" s="22"/>
+      <c r="CU4" s="22"/>
+      <c r="CV4" s="22"/>
+      <c r="CW4" s="22"/>
     </row>
-    <row r="5" spans="1:25" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:101" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1043,9 +2138,231 @@
       <c r="X5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="Y5" s="4"/>
+      <c r="Y5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AN5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AO5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AP5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AQ5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AR5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AT5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ5" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BC5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BD5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BE5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BF5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BG5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BK5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BL5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BM5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BN5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BP5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BQ5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BR5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BS5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BT5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BU5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BY5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BZ5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CB5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CC5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CD5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CF5" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="CG5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CH5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CJ5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CK5" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CL5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CM5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CN5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CO5" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CP5" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CQ5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR5" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CS5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CT5" s="22"/>
+      <c r="CU5" s="22"/>
+      <c r="CV5" s="22"/>
+      <c r="CW5" s="22"/>
     </row>
-    <row r="6" spans="1:25" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:101" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -1119,9 +2436,231 @@
       <c r="X6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Y6" s="7"/>
+      <c r="Y6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AL6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AM6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AQ6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BC6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BD6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BE6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BF6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BG6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BI6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BK6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BL6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BM6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BN6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BP6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BQ6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BR6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BS6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BT6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BU6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BW6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BY6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BZ6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CB6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CC6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CD6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE6" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CF6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CG6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CH6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CJ6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CK6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CL6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CM6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CN6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CO6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CP6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CS6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CT6" s="22"/>
+      <c r="CU6" s="22"/>
+      <c r="CV6" s="22"/>
+      <c r="CW6" s="22"/>
     </row>
-    <row r="7" spans="1:25" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:101" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1198,8 +2737,228 @@
       <c r="Y7" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="Z7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AO7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AR7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BC7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BD7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BE7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BF7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BG7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BK7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BL7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BM7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BN7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BP7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BQ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BR7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BS7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BT7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BU7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BV7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BY7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BZ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CA7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CB7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CC7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CD7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CF7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CG7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CH7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CI7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CJ7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CK7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CL7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CM7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CN7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CO7" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CP7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CS7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CT7" s="22"/>
+      <c r="CU7" s="22"/>
+      <c r="CV7" s="22"/>
+      <c r="CW7" s="22"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1276,8 +3035,228 @@
       <c r="Y8" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="Z8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC8" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AM8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AN8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AO8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AP8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BB8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BC8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BD8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BE8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BF8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BG8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BK8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BL8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BM8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BN8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BO8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BP8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BQ8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BR8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BS8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BT8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BU8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BV8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BY8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BZ8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CB8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CC8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CD8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CE8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CF8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CG8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CH8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CJ8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CK8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CL8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CM8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CN8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CO8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CP8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CR8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CS8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CT8" s="22"/>
+      <c r="CU8" s="22"/>
+      <c r="CV8" s="22"/>
+      <c r="CW8" s="22"/>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1351,7 +3330,229 @@
       <c r="X9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="Y9" s="4"/>
+      <c r="Y9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AL9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AN9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AR9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AU9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AY9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AZ9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="BA9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BC9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BD9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BE9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BF9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BG9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BH9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BJ9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BK9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BL9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BM9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BN9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BO9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BP9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BQ9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BR9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BS9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BT9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BU9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="BY9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="BZ9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CA9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CB9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CC9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="CD9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CF9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CG9" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="CH9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CI9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CJ9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CK9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CL9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CM9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CN9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CO9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CP9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ9" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CS9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="CT9" s="22"/>
+      <c r="CU9" s="22"/>
+      <c r="CV9" s="22"/>
+      <c r="CW9" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1359,11 +3560,35 @@
     <mergeCell ref="D1:Y1"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="D3:Y7 C8:Y9">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="Z3:AB9 AD4:AD8">
+    <cfRule type="cellIs" dxfId="17" priority="83" operator="equal">
       <formula>"SI"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="84" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD3:AE3 D3:Y7 AC3:AC8 C8:Y9 AC9:AD9">
+    <cfRule type="cellIs" dxfId="15" priority="87" operator="equal">
+      <formula>"SI"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="88" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE4:AE9">
+    <cfRule type="cellIs" dxfId="13" priority="81" operator="equal">
+      <formula>"SI"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="82" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF3:CW9">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+      <formula>"SI"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1383,14 +3608,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1444,11 +3669,11 @@
       </c>
       <c r="C4" s="4">
         <f>COUNTIF(Registro!D4:Y4,"SI")+COUNTIF(Registro!D4:Y4,"NO")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="4">
         <f>COUNTIF(Registro!D4:Y4,"NO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E4" s="4">
         <v>16</v>
@@ -1467,11 +3692,11 @@
       </c>
       <c r="C5" s="4">
         <f>COUNTIF(Registro!D5:Y5,"SI")+COUNTIF(Registro!D5:Y5,"NO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="4">
         <f>COUNTIF(Registro!D5:Y5,"NO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" s="4">
         <v>16</v>
@@ -1490,11 +3715,11 @@
       </c>
       <c r="C6" s="4">
         <f>COUNTIF(Registro!D6:Y6,"SI")+COUNTIF(Registro!D6:Y6,"NO")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="4">
         <f>COUNTIF(Registro!D6:Y6,"NO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="4">
         <v>16</v>
@@ -1553,11 +3778,11 @@
       </c>
       <c r="C9" s="4">
         <f>COUNTIF(Registro!D9:Y9,"SI")+COUNTIF(Registro!D9:Y9,"NO")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="4">
         <f>COUNTIF(Registro!D9:Y9,"NO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9" s="4">
         <v>16</v>
@@ -1568,14 +3793,14 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1584,4 +3809,124 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{417FC92C-5492-4C35-B239-AFF9615604B1}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:C8">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+      <formula>"SI"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+      <formula>"SI"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>